<commit_message>
Use qlHestonModel and engine
</commit_message>
<xml_diff>
--- a/tests/workbooks/test_calibratedmodel.xlsx
+++ b/tests/workbooks/test_calibratedmodel.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Sebastian\01_GitHub\sschlenkrich\QuantLibXlOil\tests\workbooks\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5135EA4C-579B-470E-9919-534391CF3851}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E1126437-59EB-41FD-A5C7-6FC047C918C8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="13905" yWindow="-20130" windowWidth="21330" windowHeight="15900" xr2:uid="{2FEFDE40-9C41-44A1-8868-8F33D5CA59CC}"/>
+    <workbookView xWindow="13530" yWindow="-19245" windowWidth="23175" windowHeight="16410" xr2:uid="{2FEFDE40-9C41-44A1-8868-8F33D5CA59CC}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
-<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
+<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
   <metadataTypes count="1">
     <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
   </metadataTypes>
@@ -61,7 +61,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="31" uniqueCount="29">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="37" uniqueCount="35">
   <si>
     <t>v0</t>
   </si>
@@ -102,9 +102,6 @@
     <t>qlSettingsSetEvaluationDate</t>
   </si>
   <si>
-    <t>tmpHestonModel</t>
-  </si>
-  <si>
     <t>qlLevenbergMarquardt</t>
   </si>
   <si>
@@ -135,9 +132,6 @@
     <t>5y</t>
   </si>
   <si>
-    <t>tmpAnalyticHestonEngine</t>
-  </si>
-  <si>
     <t>qlCalibratedModelParams</t>
   </si>
   <si>
@@ -148,6 +142,30 @@
   </si>
   <si>
     <t>qlCalibratedModelHandle</t>
+  </si>
+  <si>
+    <t>qlCalibratedModelCalibrate</t>
+  </si>
+  <si>
+    <t>qlHestonModel</t>
+  </si>
+  <si>
+    <t>qlAnalyticHestonEngine</t>
+  </si>
+  <si>
+    <t>Kappa</t>
+  </si>
+  <si>
+    <t>Rho</t>
+  </si>
+  <si>
+    <t>Sigma</t>
+  </si>
+  <si>
+    <t>Theta</t>
+  </si>
+  <si>
+    <t>V0</t>
   </si>
 </sst>
 </file>
@@ -640,25 +658,25 @@
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A18" s="1" t="s">
-        <v>13</v>
+        <v>28</v>
       </c>
       <c r="B18" t="str" cm="1">
-        <f t="array" ref="B18">_xll.tmpHestonModel(B16)</f>
+        <f t="array" ref="B18">_xll.qlHestonModel(B16)</f>
         <v>⚡[test_calibratedmodel.xlsx]Sheet1!R18C2HestonModel,A</v>
       </c>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
-        <v>24</v>
+        <v>29</v>
       </c>
       <c r="B19" t="str" cm="1">
-        <f t="array" ref="B19">_xll.tmpAnalyticHestonEngine(B18)</f>
+        <f t="array" ref="B19">_xll.qlAnalyticHestonEngine(B18)</f>
         <v>⚡[test_calibratedmodel.xlsx]Sheet1!R19C2AnalyticHestonEngine,A</v>
       </c>
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B21" t="str" cm="1">
         <f t="array" ref="B21">_xll.qlLevenbergMarquardt()</f>
@@ -667,7 +685,7 @@
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B22" t="str" cm="1">
         <f t="array" ref="B22">_xll.qlEndCriteria(100,10,0.000001,0.000001,0.000001)</f>
@@ -676,21 +694,21 @@
     </row>
     <row r="24" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
+        <v>15</v>
+      </c>
+      <c r="B24" t="s">
         <v>16</v>
-      </c>
-      <c r="B24" t="s">
-        <v>17</v>
       </c>
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.3">
       <c r="C26" t="s">
+        <v>17</v>
+      </c>
+      <c r="D26" t="s">
         <v>18</v>
       </c>
-      <c r="D26" t="s">
-        <v>19</v>
-      </c>
       <c r="E26" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
     <row r="27" spans="1:5" x14ac:dyDescent="0.3">
@@ -703,7 +721,7 @@
         <v>⚡[test_calibratedmodel.xlsx]Sheet1!R27C2HestonModelHelper,A</v>
       </c>
       <c r="C27" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="D27">
         <v>100</v>
@@ -722,7 +740,7 @@
         <v>⚡[test_calibratedmodel.xlsx]Sheet1!R28C2HestonModelHelper,A</v>
       </c>
       <c r="C28" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="D28">
         <v>80</v>
@@ -741,7 +759,7 @@
         <v>⚡[test_calibratedmodel.xlsx]Sheet1!R29C2HestonModelHelper,A</v>
       </c>
       <c r="C29" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="D29">
         <v>100</v>
@@ -760,7 +778,7 @@
         <v>⚡[test_calibratedmodel.xlsx]Sheet1!R30C2HestonModelHelper,A</v>
       </c>
       <c r="C30" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="D30">
         <v>120</v>
@@ -779,7 +797,7 @@
         <v>⚡[test_calibratedmodel.xlsx]Sheet1!R31C2HestonModelHelper,A</v>
       </c>
       <c r="C31" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D31">
         <v>100</v>
@@ -788,82 +806,100 @@
         <v>0.2</v>
       </c>
     </row>
-    <row r="33" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="B33" t="b" cm="1">
+    <row r="33" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A33" t="s">
+        <v>27</v>
+      </c>
+      <c r="B33" t="str" cm="1">
         <f t="array" ref="B33">_xll.qlCalibratedModelCalibrate(B18,B27:B31,B21,B22,,,,A27:A31)</f>
-        <v>1</v>
-      </c>
-    </row>
-    <row r="36" spans="1:2" x14ac:dyDescent="0.3">
+        <v>Error in arg 3 'optimization_method': Cannot convert '⚡[test_calibratedmodel.xlsx]Sheet1!R21C2LevenbergMarquardt,A': Expected cache string</v>
+      </c>
+    </row>
+    <row r="36" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="B36" cm="1">
         <f t="array" ref="B36:B40">_xll.qlCalibratedModelParams(B18,B33)</f>
-        <v>7.5903860839074258E-2</v>
-      </c>
-    </row>
-    <row r="37" spans="1:2" x14ac:dyDescent="0.3">
+        <v>0.04</v>
+      </c>
+      <c r="D36" cm="1">
+        <f t="array" ref="D36">_xll.qlHestonModelTheta(B18,B33)</f>
+        <v>0.04</v>
+      </c>
+      <c r="E36" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="37" spans="1:5" x14ac:dyDescent="0.3">
       <c r="B37">
-        <v>0.39716005835063128</v>
-      </c>
-    </row>
-    <row r="38" spans="1:2" x14ac:dyDescent="0.3">
+        <v>1.5</v>
+      </c>
+      <c r="D37" cm="1">
+        <f t="array" ref="D37">_xll.qlHestonModelKappa(B18,B33)</f>
+        <v>1.5</v>
+      </c>
+      <c r="E37" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="38" spans="1:5" x14ac:dyDescent="0.3">
       <c r="B38">
-        <v>1.3901714719854346</v>
-      </c>
-    </row>
-    <row r="39" spans="1:2" x14ac:dyDescent="0.3">
+        <v>0.3</v>
+      </c>
+      <c r="D38" cm="1">
+        <f t="array" ref="D38">_xll.qlHestonModelSigma(B18,B33)</f>
+        <v>0.3</v>
+      </c>
+      <c r="E38" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="39" spans="1:5" x14ac:dyDescent="0.3">
       <c r="B39">
-        <v>-0.3506856326404631</v>
-      </c>
-    </row>
-    <row r="40" spans="1:2" x14ac:dyDescent="0.3">
+        <v>-0.7</v>
+      </c>
+      <c r="D39" cm="1">
+        <f t="array" ref="D39">_xll.qlHestonModelRho(B18,B33)</f>
+        <v>-0.7</v>
+      </c>
+      <c r="E39" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="40" spans="1:5" x14ac:dyDescent="0.3">
       <c r="B40">
-        <v>0.19504877171446253</v>
-      </c>
-    </row>
-    <row r="42" spans="1:2" x14ac:dyDescent="0.3">
+        <v>0.04</v>
+      </c>
+      <c r="D40" cm="1">
+        <f t="array" ref="D40">_xll.qlHestonModelV0(B18,B33)</f>
+        <v>0.04</v>
+      </c>
+      <c r="E40" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="42" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A42" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="B42" cm="1">
-        <f t="array" ref="B42:B46">_xll.qlCalibratedModelProblemValues(B18,B33)</f>
-        <v>1.0779022980678655E-4</v>
-      </c>
-    </row>
-    <row r="43" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="B43">
-        <v>3.6377160133380237E-5</v>
-      </c>
-    </row>
-    <row r="44" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="B44">
-        <v>1.6082776976281344E-4</v>
-      </c>
-    </row>
-    <row r="45" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="B45">
-        <v>5.4411712850235827E-6</v>
-      </c>
-    </row>
-    <row r="46" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="B46">
-        <v>4.1354224029017015E-5</v>
-      </c>
-    </row>
-    <row r="48" spans="1:2" x14ac:dyDescent="0.3">
+        <f t="array" ref="B42">_xll.qlCalibratedModelProblemValues(B18,B33)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="48" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A48" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="B48" cm="1">
         <f t="array" ref="B48">_xll.qlCalibratedModelProblemValuesFunctionEvaluation(B18,B33)</f>
-        <v>20</v>
+        <v>115563376</v>
       </c>
     </row>
     <row r="50" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A50" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="B50" t="str" cm="1">
         <f t="array" ref="B50">_xll.qlCalibratedModelHandle(B18)</f>

</xml_diff>